<commit_message>
Add Specimens as fourth grouping output
</commit_message>
<xml_diff>
--- a/r-material-examined/data/danwinnie export for SRNP Type_AME complete.xlsx
+++ b/r-material-examined/data/danwinnie export for SRNP Type_AME complete.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilydarling/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E80B0C47-F9AF-4F31-8BCF-121A17830B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D4B478-6956-1C43-8421-4472BA54A478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4300" yWindow="-21000" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="224">
   <si>
     <t>sort</t>
   </si>
@@ -807,9 +807,6 @@
   <si>
     <t>14-SRNP-71696</t>
   </si>
-  <si>
-    <t>Material</t>
-  </si>
 </sst>
 </file>
 
@@ -819,7 +816,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="dd/mmm/yyyy"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1194,11 +1191,11 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1558,21 +1555,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AX14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="19.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="6" max="6" width="19.5" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.1640625" customWidth="1"/>
     <col min="16" max="16" width="41" customWidth="1"/>
-    <col min="17" max="17" width="15.140625" customWidth="1"/>
-    <col min="18" max="18" width="15.85546875" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" customWidth="1"/>
-    <col min="37" max="37" width="12.85546875" customWidth="1"/>
-    <col min="49" max="49" width="20.7109375" customWidth="1"/>
-    <col min="50" max="50" width="24.140625" customWidth="1"/>
+    <col min="17" max="17" width="15.1640625" customWidth="1"/>
+    <col min="18" max="18" width="15.83203125" customWidth="1"/>
+    <col min="36" max="36" width="12.5" customWidth="1"/>
+    <col min="37" max="37" width="12.83203125" customWidth="1"/>
+    <col min="49" max="49" width="20.6640625" customWidth="1"/>
+    <col min="50" max="50" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" ht="135">
+    <row r="1" spans="1:50" ht="112" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1712,7 +1709,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="2" spans="1:50" s="62" customFormat="1" ht="60">
+    <row r="2" spans="1:50" s="62" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="34">
         <v>3118</v>
       </c>
@@ -1830,7 +1827,7 @@
       <c r="AW2" s="56"/>
       <c r="AX2" s="42"/>
     </row>
-    <row r="3" spans="1:50">
+    <row r="3" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A3" s="34">
         <v>3117</v>
       </c>
@@ -1946,7 +1943,7 @@
       <c r="AW3" s="56"/>
       <c r="AX3" s="42"/>
     </row>
-    <row r="4" spans="1:50">
+    <row r="4" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A4" s="18">
         <v>14</v>
       </c>
@@ -1971,9 +1968,7 @@
       <c r="J4" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="K4" s="58" t="s">
-        <v>224</v>
-      </c>
+      <c r="K4" s="58"/>
       <c r="L4" s="19"/>
       <c r="M4" s="20" t="s">
         <v>52</v>
@@ -2046,7 +2041,7 @@
       <c r="AW4" s="56"/>
       <c r="AX4" s="19"/>
     </row>
-    <row r="5" spans="1:50" ht="75">
+    <row r="5" spans="1:50" ht="80" x14ac:dyDescent="0.2">
       <c r="A5" s="34">
         <v>16</v>
       </c>
@@ -2158,7 +2153,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:50">
+    <row r="6" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A6" s="18">
         <v>13</v>
       </c>
@@ -2266,7 +2261,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="7" spans="1:50">
+    <row r="7" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A7" s="18">
         <v>15</v>
       </c>
@@ -2378,7 +2373,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:50">
+    <row r="8" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A8" s="18">
         <v>12</v>
       </c>
@@ -2486,7 +2481,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:50">
+    <row r="9" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A9" s="18">
         <v>2944</v>
       </c>
@@ -2589,7 +2584,7 @@
       <c r="AT9" s="19"/>
       <c r="AX9" s="19"/>
     </row>
-    <row r="10" spans="1:50">
+    <row r="10" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A10" s="18">
         <v>3116</v>
       </c>
@@ -2692,7 +2687,7 @@
       <c r="AT10" s="19"/>
       <c r="AX10" s="20"/>
     </row>
-    <row r="11" spans="1:50">
+    <row r="11" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A11" s="18">
         <v>193</v>
       </c>
@@ -2721,9 +2716,7 @@
       <c r="J11" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="K11" s="58" t="s">
-        <v>224</v>
-      </c>
+      <c r="K11" s="58"/>
       <c r="L11" s="19"/>
       <c r="M11" s="20" t="s">
         <v>161</v>
@@ -2803,7 +2796,7 @@
       <c r="AT11" s="19"/>
       <c r="AX11" s="19"/>
     </row>
-    <row r="12" spans="1:50" ht="30">
+    <row r="12" spans="1:50" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="18">
         <v>3121</v>
       </c>
@@ -2832,9 +2825,7 @@
       <c r="J12" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="58" t="s">
-        <v>224</v>
-      </c>
+      <c r="K12" s="58"/>
       <c r="L12" s="19" t="s">
         <v>195</v>
       </c>
@@ -2898,7 +2889,7 @@
       <c r="AT12" s="19"/>
       <c r="AX12" s="26"/>
     </row>
-    <row r="13" spans="1:50">
+    <row r="13" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A13" s="18">
         <v>2877</v>
       </c>
@@ -2923,9 +2914,7 @@
       <c r="J13" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="58" t="s">
-        <v>224</v>
-      </c>
+      <c r="K13" s="58"/>
       <c r="L13" s="19"/>
       <c r="M13" s="20" t="s">
         <v>52</v>
@@ -2993,7 +2982,7 @@
       <c r="AT13" s="19"/>
       <c r="AX13" s="19"/>
     </row>
-    <row r="14" spans="1:50">
+    <row r="14" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A14" s="51"/>
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>

</xml_diff>